<commit_message>
Yaml configurations for main training pipeline
</commit_message>
<xml_diff>
--- a/labeling_bbch_iso_dates.xlsx
+++ b/labeling_bbch_iso_dates.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ASUS\Desktop\Ders\blg521\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD804091-6EBC-4AE3-A0E3-9FF15007FD8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5F885CD-C54B-4600-AEF7-D0A4FF2D377D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1116" yWindow="1116" windowWidth="18588" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="labels" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="51">
   <si>
     <t>ID</t>
   </si>
@@ -186,9 +186,6 @@
   </si>
   <si>
     <t>01.17</t>
-  </si>
-  <si>
-    <t>21.06</t>
   </si>
 </sst>
 </file>
@@ -365,7 +362,7 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -451,7 +448,6 @@
     <xf numFmtId="49" fontId="12" fillId="8" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="12" fillId="8" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -630,7 +626,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:W36"/>
+  <dimension ref="A1:W35"/>
   <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3" customWidth="1"/>
@@ -725,9 +721,6 @@
       <c r="V1" t="s">
         <v>20</v>
       </c>
-      <c r="W1" t="s">
-        <v>3</v>
-      </c>
     </row>
     <row r="2" spans="1:23" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A2" s="26">
@@ -792,7 +785,7 @@
         <v>24</v>
       </c>
       <c r="S2" s="5">
-        <f t="shared" ref="S2:S26" si="4">SUM(L2:R2)</f>
+        <f t="shared" ref="S2:S25" si="4">SUM(L2:R2)</f>
         <v>187</v>
       </c>
       <c r="T2" s="29">
@@ -837,31 +830,31 @@
         <v>42894</v>
       </c>
       <c r="L3" s="5">
-        <f t="shared" ref="L3:L26" si="5">E3-D3</f>
+        <f t="shared" ref="L3:L25" si="5">E3-D3</f>
         <v>36</v>
       </c>
       <c r="M3" s="5">
-        <f t="shared" ref="M3:M26" si="6">F3-E3</f>
+        <f t="shared" ref="M3:M25" si="6">F3-E3</f>
         <v>26</v>
       </c>
       <c r="N3" s="5">
-        <f t="shared" ref="N3:N26" si="7">G3-F3</f>
+        <f t="shared" ref="N3:N25" si="7">G3-F3</f>
         <v>48</v>
       </c>
       <c r="O3" s="7">
-        <f t="shared" ref="O3:O26" si="8">H3-G3</f>
+        <f t="shared" ref="O3:O25" si="8">H3-G3</f>
         <v>33</v>
       </c>
       <c r="P3" s="5">
-        <f t="shared" ref="P3:P26" si="9">I3-H3</f>
+        <f t="shared" ref="P3:P25" si="9">I3-H3</f>
         <v>11</v>
       </c>
       <c r="Q3" s="5">
-        <f t="shared" ref="Q3:Q26" si="10">J3-I3</f>
+        <f t="shared" ref="Q3:Q25" si="10">J3-I3</f>
         <v>29</v>
       </c>
       <c r="R3" s="5">
-        <f t="shared" ref="R3:R26" si="11">K3-J3</f>
+        <f t="shared" ref="R3:R25" si="11">K3-J3</f>
         <v>21</v>
       </c>
       <c r="S3" s="5">
@@ -874,13 +867,12 @@
       <c r="U3" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="W3" s="31">
-        <f>SUM(S2:S3)</f>
-        <v>391</v>
-      </c>
+      <c r="W3" s="31"/>
     </row>
     <row r="4" spans="1:23" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A4" s="26"/>
+      <c r="A4" s="26">
+        <v>3</v>
+      </c>
       <c r="B4" s="30" t="s">
         <v>50</v>
       </c>
@@ -950,8 +942,8 @@
       <c r="W4" s="31"/>
     </row>
     <row r="5" spans="1:23" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A5" s="1">
-        <v>3</v>
+      <c r="A5" s="26">
+        <v>4</v>
       </c>
       <c r="B5" s="14" t="s">
         <v>6</v>
@@ -1024,7 +1016,7 @@
     </row>
     <row r="6" spans="1:23" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A6" s="26">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B6" s="14" t="s">
         <v>8</v>
@@ -1097,7 +1089,7 @@
     </row>
     <row r="7" spans="1:23" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A7" s="26">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B7" s="14" t="s">
         <v>8</v>
@@ -1169,8 +1161,8 @@
       </c>
     </row>
     <row r="8" spans="1:23" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A8" s="1">
-        <v>6</v>
+      <c r="A8" s="26">
+        <v>7</v>
       </c>
       <c r="B8" s="14" t="s">
         <v>9</v>
@@ -1243,7 +1235,7 @@
     </row>
     <row r="9" spans="1:23" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A9" s="26">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B9" s="14" t="s">
         <v>10</v>
@@ -1316,7 +1308,7 @@
     </row>
     <row r="10" spans="1:23" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A10" s="26">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B10" s="14" t="s">
         <v>11</v>
@@ -1387,14 +1379,11 @@
       <c r="U10" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="W10" s="31">
-        <f>SUM(S5:S10)</f>
-        <v>1289</v>
-      </c>
+      <c r="W10" s="31"/>
     </row>
     <row r="11" spans="1:23" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A11" s="1">
-        <v>9</v>
+      <c r="A11" s="26">
+        <v>10</v>
       </c>
       <c r="B11" s="14" t="s">
         <v>12</v>
@@ -1467,7 +1456,7 @@
     </row>
     <row r="12" spans="1:23" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A12" s="26">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B12" s="14" t="s">
         <v>13</v>
@@ -1543,7 +1532,7 @@
     </row>
     <row r="13" spans="1:23" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A13" s="26">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B13" s="14" t="s">
         <v>13</v>
@@ -1618,8 +1607,8 @@
       </c>
     </row>
     <row r="14" spans="1:23" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A14" s="1">
-        <v>12</v>
+      <c r="A14" s="26">
+        <v>13</v>
       </c>
       <c r="B14" s="14" t="s">
         <v>14</v>
@@ -1693,457 +1682,515 @@
         <v>42</v>
       </c>
     </row>
-    <row r="15" spans="1:23" s="39" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A15" s="33"/>
+    <row r="15" spans="1:23" s="38" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A15" s="26">
+        <v>14</v>
+      </c>
       <c r="B15" s="32" t="s">
         <v>43</v>
       </c>
-      <c r="C15" s="34">
+      <c r="C15" s="33">
         <v>2016</v>
       </c>
-      <c r="D15" s="35">
+      <c r="D15" s="34">
         <v>42667</v>
       </c>
-      <c r="E15" s="35">
+      <c r="E15" s="34">
         <v>42693</v>
       </c>
-      <c r="F15" s="35">
+      <c r="F15" s="34">
         <v>42805</v>
       </c>
-      <c r="G15" s="35">
+      <c r="G15" s="34">
         <v>42826</v>
       </c>
-      <c r="H15" s="35">
+      <c r="H15" s="34">
         <v>42881</v>
       </c>
-      <c r="I15" s="35">
+      <c r="I15" s="34">
         <v>42892</v>
       </c>
-      <c r="J15" s="35">
+      <c r="J15" s="34">
         <v>42904</v>
       </c>
-      <c r="K15" s="35">
+      <c r="K15" s="34">
         <v>42931</v>
       </c>
-      <c r="L15" s="36">
+      <c r="L15" s="35">
         <f t="shared" ref="L15:N19" si="21">E15-D15</f>
         <v>26</v>
       </c>
-      <c r="M15" s="36">
+      <c r="M15" s="35">
         <f t="shared" si="21"/>
         <v>112</v>
       </c>
-      <c r="N15" s="36">
+      <c r="N15" s="35">
         <f t="shared" si="21"/>
         <v>21</v>
       </c>
-      <c r="O15" s="37">
+      <c r="O15" s="36">
         <f t="shared" si="8"/>
         <v>55</v>
       </c>
-      <c r="P15" s="36">
+      <c r="P15" s="35">
         <f t="shared" si="9"/>
         <v>11</v>
       </c>
-      <c r="Q15" s="36">
+      <c r="Q15" s="35">
         <f t="shared" si="10"/>
         <v>12</v>
       </c>
-      <c r="R15" s="36">
+      <c r="R15" s="35">
         <f t="shared" si="11"/>
         <v>27</v>
       </c>
-      <c r="S15" s="36">
+      <c r="S15" s="35">
         <f t="shared" si="4"/>
         <v>264</v>
       </c>
-      <c r="T15" s="38">
+      <c r="T15" s="37">
         <v>1</v>
       </c>
-      <c r="U15" s="38" t="s">
+      <c r="U15" s="37" t="s">
         <v>7</v>
       </c>
-      <c r="V15" s="39" t="s">
+      <c r="V15" s="38" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="16" spans="1:23" s="39" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A16" s="33"/>
+    <row r="16" spans="1:23" s="38" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A16" s="26">
+        <v>15</v>
+      </c>
       <c r="B16" s="32" t="s">
         <v>45</v>
       </c>
-      <c r="C16" s="34">
+      <c r="C16" s="33">
         <v>2013</v>
       </c>
-      <c r="D16" s="35">
+      <c r="D16" s="34">
         <v>41581</v>
       </c>
-      <c r="E16" s="35">
+      <c r="E16" s="34">
         <v>41605</v>
       </c>
-      <c r="F16" s="35">
+      <c r="F16" s="34">
         <v>41663</v>
       </c>
-      <c r="G16" s="35">
+      <c r="G16" s="34">
         <v>41705</v>
       </c>
-      <c r="H16" s="35">
+      <c r="H16" s="34">
         <v>41761</v>
       </c>
-      <c r="I16" s="35">
+      <c r="I16" s="34">
         <v>41784</v>
       </c>
-      <c r="J16" s="35">
+      <c r="J16" s="34">
         <v>41797</v>
       </c>
-      <c r="K16" s="35">
+      <c r="K16" s="34">
         <v>41810</v>
       </c>
-      <c r="L16" s="36">
+      <c r="L16" s="35">
         <f t="shared" si="21"/>
         <v>24</v>
       </c>
-      <c r="M16" s="36">
+      <c r="M16" s="35">
         <f t="shared" si="21"/>
         <v>58</v>
       </c>
-      <c r="N16" s="36">
+      <c r="N16" s="35">
         <f t="shared" si="21"/>
         <v>42</v>
       </c>
-      <c r="O16" s="37">
+      <c r="O16" s="36">
         <f t="shared" si="8"/>
         <v>56</v>
       </c>
-      <c r="P16" s="36">
+      <c r="P16" s="35">
         <f t="shared" si="9"/>
         <v>23</v>
       </c>
-      <c r="Q16" s="36">
+      <c r="Q16" s="35">
         <f t="shared" si="10"/>
         <v>13</v>
       </c>
-      <c r="R16" s="36">
+      <c r="R16" s="35">
         <f t="shared" si="11"/>
         <v>13</v>
       </c>
-      <c r="S16" s="36">
+      <c r="S16" s="35">
         <f t="shared" si="4"/>
         <v>229</v>
       </c>
       <c r="T16" s="8">
         <v>1</v>
       </c>
-      <c r="U16" s="38" t="s">
+      <c r="U16" s="37" t="s">
         <v>7</v>
       </c>
-      <c r="V16" s="39" t="s">
+      <c r="V16" s="38" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="17" spans="1:23" s="39" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A17" s="33"/>
+    <row r="17" spans="1:23" s="38" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A17" s="26">
+        <v>16</v>
+      </c>
       <c r="B17" s="32" t="s">
         <v>46</v>
       </c>
-      <c r="C17" s="34">
+      <c r="C17" s="33">
         <v>2014</v>
       </c>
-      <c r="D17" s="35">
+      <c r="D17" s="34">
         <v>41925</v>
       </c>
-      <c r="E17" s="35">
+      <c r="E17" s="34">
         <v>41997</v>
       </c>
-      <c r="F17" s="35">
+      <c r="F17" s="34">
         <v>42065</v>
       </c>
-      <c r="G17" s="35">
+      <c r="G17" s="34">
         <v>42083</v>
       </c>
-      <c r="H17" s="35">
+      <c r="H17" s="34">
         <v>42131</v>
       </c>
-      <c r="I17" s="35">
+      <c r="I17" s="34">
         <v>42144</v>
       </c>
-      <c r="J17" s="35">
+      <c r="J17" s="34">
         <v>42160</v>
       </c>
-      <c r="K17" s="35">
+      <c r="K17" s="34">
         <v>42199</v>
       </c>
-      <c r="L17" s="36">
+      <c r="L17" s="35">
         <f t="shared" si="21"/>
         <v>72</v>
       </c>
-      <c r="M17" s="36">
+      <c r="M17" s="35">
         <f t="shared" si="21"/>
         <v>68</v>
       </c>
-      <c r="N17" s="36">
+      <c r="N17" s="35">
         <f t="shared" si="21"/>
         <v>18</v>
       </c>
-      <c r="O17" s="37">
+      <c r="O17" s="36">
         <f t="shared" si="8"/>
         <v>48</v>
       </c>
-      <c r="P17" s="36">
+      <c r="P17" s="35">
         <f t="shared" si="9"/>
         <v>13</v>
       </c>
-      <c r="Q17" s="36">
+      <c r="Q17" s="35">
         <f t="shared" si="10"/>
         <v>16</v>
       </c>
-      <c r="R17" s="36">
+      <c r="R17" s="35">
         <f t="shared" si="11"/>
         <v>39</v>
       </c>
-      <c r="S17" s="36">
+      <c r="S17" s="35">
         <f t="shared" si="4"/>
         <v>274</v>
       </c>
       <c r="T17" s="8">
         <v>1</v>
       </c>
-      <c r="U17" s="38" t="s">
+      <c r="U17" s="37" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="18" spans="1:23" s="39" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A18" s="33"/>
+    <row r="18" spans="1:23" s="38" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A18" s="26">
+        <v>17</v>
+      </c>
       <c r="B18" s="32" t="s">
         <v>48</v>
       </c>
-      <c r="C18" s="34">
+      <c r="C18" s="33">
         <v>2016</v>
       </c>
-      <c r="D18" s="35">
+      <c r="D18" s="34">
         <v>42665</v>
       </c>
-      <c r="E18" s="35">
+      <c r="E18" s="34">
         <v>42793</v>
       </c>
-      <c r="F18" s="35">
+      <c r="F18" s="34">
         <v>42818</v>
       </c>
-      <c r="G18" s="35">
+      <c r="G18" s="34">
         <v>42844</v>
       </c>
-      <c r="H18" s="35">
+      <c r="H18" s="34">
         <v>42892</v>
       </c>
-      <c r="I18" s="35">
+      <c r="I18" s="34">
         <v>42904</v>
       </c>
-      <c r="J18" s="35">
+      <c r="J18" s="34">
         <v>42930</v>
       </c>
-      <c r="K18" s="35">
+      <c r="K18" s="34">
         <v>42951</v>
       </c>
-      <c r="L18" s="36">
+      <c r="L18" s="35">
         <f t="shared" si="21"/>
         <v>128</v>
       </c>
-      <c r="M18" s="36">
+      <c r="M18" s="35">
         <f t="shared" si="21"/>
         <v>25</v>
       </c>
-      <c r="N18" s="36">
+      <c r="N18" s="35">
         <f t="shared" si="21"/>
         <v>26</v>
       </c>
-      <c r="O18" s="37">
+      <c r="O18" s="36">
         <f t="shared" si="8"/>
         <v>48</v>
       </c>
-      <c r="P18" s="36">
+      <c r="P18" s="35">
         <f t="shared" si="9"/>
         <v>12</v>
       </c>
-      <c r="Q18" s="36">
+      <c r="Q18" s="35">
         <f t="shared" si="10"/>
         <v>26</v>
       </c>
-      <c r="R18" s="36">
+      <c r="R18" s="35">
         <f t="shared" si="11"/>
         <v>21</v>
       </c>
-      <c r="S18" s="36">
+      <c r="S18" s="35">
         <f t="shared" si="4"/>
         <v>286</v>
       </c>
       <c r="T18" s="8">
         <v>1</v>
       </c>
-      <c r="U18" s="38" t="s">
+      <c r="U18" s="37" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="19" spans="1:23" s="39" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A19" s="33"/>
+    <row r="19" spans="1:23" s="38" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A19" s="26">
+        <v>18</v>
+      </c>
       <c r="B19" s="32" t="s">
         <v>49</v>
       </c>
-      <c r="C19" s="34">
+      <c r="C19" s="33">
         <v>2013</v>
       </c>
-      <c r="D19" s="35">
+      <c r="D19" s="34">
         <v>41598</v>
       </c>
-      <c r="E19" s="35">
+      <c r="E19" s="34">
         <v>41612</v>
       </c>
-      <c r="F19" s="35">
+      <c r="F19" s="34">
         <v>41689</v>
       </c>
-      <c r="G19" s="35">
+      <c r="G19" s="34">
         <v>41705</v>
       </c>
-      <c r="H19" s="35">
+      <c r="H19" s="34">
         <v>41757</v>
       </c>
-      <c r="I19" s="35">
+      <c r="I19" s="34">
         <v>41774</v>
       </c>
-      <c r="J19" s="35">
+      <c r="J19" s="34">
         <v>41787</v>
       </c>
-      <c r="K19" s="35">
+      <c r="K19" s="34">
         <v>41808</v>
       </c>
-      <c r="L19" s="36">
+      <c r="L19" s="35">
         <f t="shared" si="21"/>
         <v>14</v>
       </c>
-      <c r="M19" s="36">
+      <c r="M19" s="35">
         <f t="shared" si="21"/>
         <v>77</v>
       </c>
-      <c r="N19" s="36">
+      <c r="N19" s="35">
         <f t="shared" si="21"/>
         <v>16</v>
       </c>
-      <c r="O19" s="37">
+      <c r="O19" s="36">
         <f t="shared" si="8"/>
         <v>52</v>
       </c>
-      <c r="P19" s="36">
+      <c r="P19" s="35">
         <f t="shared" si="9"/>
         <v>17</v>
       </c>
-      <c r="Q19" s="36">
+      <c r="Q19" s="35">
         <f t="shared" si="10"/>
         <v>13</v>
       </c>
-      <c r="R19" s="36">
+      <c r="R19" s="35">
         <f t="shared" si="11"/>
         <v>21</v>
       </c>
-      <c r="S19" s="36">
+      <c r="S19" s="35">
         <f t="shared" si="4"/>
         <v>210</v>
       </c>
       <c r="T19" s="8">
         <v>1</v>
       </c>
-      <c r="U19" s="38" t="s">
+      <c r="U19" s="37" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="20" spans="1:23" s="39" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A20" s="33"/>
-      <c r="B20" s="32" t="s">
-        <v>51</v>
-      </c>
-      <c r="C20" s="34"/>
-      <c r="D20" s="35"/>
-      <c r="E20" s="35"/>
-      <c r="F20" s="35"/>
-      <c r="G20" s="35"/>
-      <c r="H20" s="35"/>
-      <c r="I20" s="35"/>
-      <c r="J20" s="35"/>
-      <c r="K20" s="35"/>
-      <c r="L20" s="36"/>
-      <c r="M20" s="36"/>
-      <c r="N20" s="36"/>
-      <c r="O20" s="37"/>
-      <c r="P20" s="36"/>
-      <c r="Q20" s="36"/>
-      <c r="R20" s="36"/>
-      <c r="S20" s="36"/>
-      <c r="T20" s="8"/>
-      <c r="U20" s="38"/>
+    <row r="20" spans="1:23" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A20" s="26">
+        <v>19</v>
+      </c>
+      <c r="B20" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="C20" s="15">
+        <v>2016</v>
+      </c>
+      <c r="D20" s="21">
+        <v>42662</v>
+      </c>
+      <c r="E20" s="21">
+        <v>42777</v>
+      </c>
+      <c r="F20" s="21">
+        <v>42827</v>
+      </c>
+      <c r="G20" s="21">
+        <v>42860</v>
+      </c>
+      <c r="H20" s="21">
+        <v>42877</v>
+      </c>
+      <c r="I20" s="21">
+        <v>42884</v>
+      </c>
+      <c r="J20" s="21">
+        <v>42909</v>
+      </c>
+      <c r="K20" s="21">
+        <v>42939</v>
+      </c>
+      <c r="L20" s="5">
+        <f t="shared" si="5"/>
+        <v>115</v>
+      </c>
+      <c r="M20" s="5">
+        <f t="shared" si="6"/>
+        <v>50</v>
+      </c>
+      <c r="N20" s="5">
+        <f t="shared" si="7"/>
+        <v>33</v>
+      </c>
+      <c r="O20" s="7">
+        <f t="shared" si="8"/>
+        <v>17</v>
+      </c>
+      <c r="P20" s="5">
+        <f t="shared" si="9"/>
+        <v>7</v>
+      </c>
+      <c r="Q20" s="5">
+        <f t="shared" si="10"/>
+        <v>25</v>
+      </c>
+      <c r="R20" s="5">
+        <f t="shared" si="11"/>
+        <v>30</v>
+      </c>
+      <c r="S20" s="5">
+        <f t="shared" si="4"/>
+        <v>277</v>
+      </c>
+      <c r="T20" s="8">
+        <v>1</v>
+      </c>
+      <c r="U20" s="8" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="21" spans="1:23" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A21" s="26">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="B21" s="16" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C21" s="15">
         <v>2016</v>
       </c>
       <c r="D21" s="21">
-        <v>42662</v>
+        <v>42642</v>
       </c>
       <c r="E21" s="21">
-        <v>42777</v>
+        <v>42771</v>
       </c>
       <c r="F21" s="21">
-        <v>42827</v>
+        <v>42826</v>
       </c>
       <c r="G21" s="21">
-        <v>42860</v>
+        <v>42856</v>
       </c>
       <c r="H21" s="21">
-        <v>42877</v>
+        <v>42878</v>
       </c>
       <c r="I21" s="21">
-        <v>42884</v>
+        <v>42889</v>
       </c>
       <c r="J21" s="21">
-        <v>42909</v>
+        <v>42918</v>
       </c>
       <c r="K21" s="21">
-        <v>42939</v>
+        <v>42937</v>
       </c>
       <c r="L21" s="5">
         <f t="shared" si="5"/>
-        <v>115</v>
+        <v>129</v>
       </c>
       <c r="M21" s="5">
         <f t="shared" si="6"/>
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="N21" s="5">
         <f t="shared" si="7"/>
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="O21" s="7">
         <f t="shared" si="8"/>
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="P21" s="5">
         <f t="shared" si="9"/>
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="Q21" s="5">
         <f t="shared" si="10"/>
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="R21" s="5">
         <f t="shared" si="11"/>
-        <v>30</v>
+        <v>19</v>
       </c>
       <c r="S21" s="5">
         <f t="shared" si="4"/>
-        <v>277</v>
+        <v>295</v>
       </c>
       <c r="T21" s="8">
         <v>1</v>
@@ -2151,72 +2198,75 @@
       <c r="U21" s="8" t="s">
         <v>7</v>
       </c>
+      <c r="V21" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row r="22" spans="1:23" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A22" s="26">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="B22" s="16" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C22" s="15">
         <v>2016</v>
       </c>
       <c r="D22" s="21">
-        <v>42642</v>
+        <v>42688</v>
       </c>
       <c r="E22" s="21">
-        <v>42771</v>
+        <v>42707</v>
       </c>
       <c r="F22" s="21">
-        <v>42826</v>
+        <v>42773</v>
       </c>
       <c r="G22" s="21">
-        <v>42856</v>
+        <v>42807</v>
       </c>
       <c r="H22" s="21">
-        <v>42878</v>
+        <v>42858</v>
       </c>
       <c r="I22" s="21">
-        <v>42889</v>
+        <v>42872</v>
       </c>
       <c r="J22" s="21">
-        <v>42918</v>
+        <v>42890</v>
       </c>
       <c r="K22" s="21">
-        <v>42937</v>
+        <v>42908</v>
       </c>
       <c r="L22" s="5">
         <f t="shared" si="5"/>
-        <v>129</v>
+        <v>19</v>
       </c>
       <c r="M22" s="5">
         <f t="shared" si="6"/>
-        <v>55</v>
+        <v>66</v>
       </c>
       <c r="N22" s="5">
         <f t="shared" si="7"/>
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="O22" s="7">
         <f t="shared" si="8"/>
-        <v>22</v>
+        <v>51</v>
       </c>
       <c r="P22" s="5">
         <f t="shared" si="9"/>
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="Q22" s="5">
         <f t="shared" si="10"/>
-        <v>29</v>
+        <v>18</v>
       </c>
       <c r="R22" s="5">
         <f t="shared" si="11"/>
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="S22" s="5">
         <f t="shared" si="4"/>
-        <v>295</v>
+        <v>220</v>
       </c>
       <c r="T22" s="8">
         <v>1</v>
@@ -2224,16 +2274,14 @@
       <c r="U22" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="V22" t="s">
-        <v>41</v>
-      </c>
+      <c r="W22" s="31"/>
     </row>
     <row r="23" spans="1:23" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A23" s="1">
-        <v>15</v>
+      <c r="A23" s="26">
+        <v>22</v>
       </c>
       <c r="B23" s="16" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C23" s="15">
         <v>2016</v>
@@ -2242,57 +2290,57 @@
         <v>42688</v>
       </c>
       <c r="E23" s="21">
-        <v>42707</v>
+        <v>42719</v>
       </c>
       <c r="F23" s="21">
-        <v>42773</v>
+        <v>42786</v>
       </c>
       <c r="G23" s="21">
-        <v>42807</v>
+        <v>42811</v>
       </c>
       <c r="H23" s="21">
-        <v>42858</v>
+        <v>42852</v>
       </c>
       <c r="I23" s="21">
-        <v>42872</v>
+        <v>42875</v>
       </c>
       <c r="J23" s="21">
-        <v>42890</v>
+        <v>42891</v>
       </c>
       <c r="K23" s="21">
-        <v>42908</v>
+        <v>42906</v>
       </c>
       <c r="L23" s="5">
         <f t="shared" si="5"/>
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="M23" s="5">
         <f t="shared" si="6"/>
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="N23" s="5">
         <f t="shared" si="7"/>
-        <v>34</v>
+        <v>25</v>
       </c>
       <c r="O23" s="7">
         <f t="shared" si="8"/>
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="P23" s="5">
         <f t="shared" si="9"/>
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="Q23" s="5">
         <f t="shared" si="10"/>
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="R23" s="5">
         <f t="shared" si="11"/>
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="S23" s="5">
         <f t="shared" si="4"/>
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="T23" s="8">
         <v>1</v>
@@ -2300,76 +2348,72 @@
       <c r="U23" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="W23" s="31">
-        <f>SUM(S23:S25)</f>
-        <v>630</v>
-      </c>
     </row>
     <row r="24" spans="1:23" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A24" s="26">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="B24" s="16" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C24" s="15">
-        <v>2016</v>
+        <v>2013</v>
       </c>
       <c r="D24" s="21">
-        <v>42688</v>
+        <v>41610</v>
       </c>
       <c r="E24" s="21">
-        <v>42719</v>
+        <v>41634</v>
       </c>
       <c r="F24" s="21">
-        <v>42786</v>
+        <v>41668</v>
       </c>
       <c r="G24" s="21">
-        <v>42811</v>
+        <v>41709</v>
       </c>
       <c r="H24" s="21">
-        <v>42852</v>
+        <v>41745</v>
       </c>
       <c r="I24" s="21">
-        <v>42875</v>
+        <v>41764</v>
       </c>
       <c r="J24" s="21">
-        <v>42891</v>
+        <v>41793</v>
       </c>
       <c r="K24" s="21">
-        <v>42906</v>
+        <v>41802</v>
       </c>
       <c r="L24" s="5">
         <f t="shared" si="5"/>
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="M24" s="5">
         <f t="shared" si="6"/>
-        <v>67</v>
+        <v>34</v>
       </c>
       <c r="N24" s="5">
         <f t="shared" si="7"/>
-        <v>25</v>
+        <v>41</v>
       </c>
       <c r="O24" s="7">
         <f t="shared" si="8"/>
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="P24" s="5">
         <f t="shared" si="9"/>
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="Q24" s="5">
         <f t="shared" si="10"/>
-        <v>16</v>
+        <v>29</v>
       </c>
       <c r="R24" s="5">
         <f t="shared" si="11"/>
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="S24" s="5">
         <f t="shared" si="4"/>
-        <v>218</v>
+        <v>192</v>
       </c>
       <c r="T24" s="8">
         <v>1</v>
@@ -2378,55 +2422,55 @@
         <v>7</v>
       </c>
     </row>
-    <row r="25" spans="1:23" ht="13.8" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:23" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A25" s="26">
-        <v>17</v>
-      </c>
-      <c r="B25" s="16" t="s">
+        <v>24</v>
+      </c>
+      <c r="B25" s="18" t="s">
         <v>19</v>
       </c>
-      <c r="C25" s="15">
-        <v>2013</v>
-      </c>
-      <c r="D25" s="21">
-        <v>41610</v>
-      </c>
-      <c r="E25" s="21">
-        <v>41634</v>
-      </c>
-      <c r="F25" s="21">
-        <v>41668</v>
-      </c>
-      <c r="G25" s="21">
-        <v>41709</v>
-      </c>
-      <c r="H25" s="21">
-        <v>41745</v>
-      </c>
-      <c r="I25" s="21">
-        <v>41764</v>
-      </c>
-      <c r="J25" s="21">
-        <v>41793</v>
-      </c>
-      <c r="K25" s="21">
-        <v>41802</v>
+      <c r="C25" s="17">
+        <v>2016</v>
+      </c>
+      <c r="D25" s="22">
+        <v>42703</v>
+      </c>
+      <c r="E25" s="22">
+        <v>42730</v>
+      </c>
+      <c r="F25" s="22">
+        <v>42783</v>
+      </c>
+      <c r="G25" s="22">
+        <v>42814</v>
+      </c>
+      <c r="H25" s="22">
+        <v>42853</v>
+      </c>
+      <c r="I25" s="22">
+        <v>42872</v>
+      </c>
+      <c r="J25" s="22">
+        <v>42887</v>
+      </c>
+      <c r="K25" s="23">
+        <v>42898</v>
       </c>
       <c r="L25" s="5">
         <f t="shared" si="5"/>
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="M25" s="5">
         <f t="shared" si="6"/>
-        <v>34</v>
+        <v>53</v>
       </c>
       <c r="N25" s="5">
         <f t="shared" si="7"/>
-        <v>41</v>
+        <v>31</v>
       </c>
       <c r="O25" s="7">
         <f t="shared" si="8"/>
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="P25" s="5">
         <f t="shared" si="9"/>
@@ -2434,15 +2478,15 @@
       </c>
       <c r="Q25" s="5">
         <f t="shared" si="10"/>
-        <v>29</v>
+        <v>15</v>
       </c>
       <c r="R25" s="5">
         <f t="shared" si="11"/>
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="S25" s="5">
         <f t="shared" si="4"/>
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="T25" s="8">
         <v>1</v>
@@ -2450,120 +2494,50 @@
       <c r="U25" s="8" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="26" spans="1:23" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A26" s="1">
-        <v>18</v>
-      </c>
-      <c r="B26" s="18" t="s">
-        <v>19</v>
-      </c>
-      <c r="C26" s="17">
-        <v>2016</v>
-      </c>
-      <c r="D26" s="22">
-        <v>42703</v>
-      </c>
-      <c r="E26" s="22">
-        <v>42730</v>
-      </c>
-      <c r="F26" s="22">
-        <v>42783</v>
-      </c>
-      <c r="G26" s="22">
-        <v>42814</v>
-      </c>
-      <c r="H26" s="22">
-        <v>42853</v>
-      </c>
-      <c r="I26" s="22">
-        <v>42872</v>
-      </c>
-      <c r="J26" s="22">
-        <v>42887</v>
-      </c>
-      <c r="K26" s="23">
-        <v>42898</v>
-      </c>
-      <c r="L26" s="5">
-        <f t="shared" si="5"/>
-        <v>27</v>
-      </c>
-      <c r="M26" s="5">
-        <f t="shared" si="6"/>
-        <v>53</v>
-      </c>
-      <c r="N26" s="5">
-        <f t="shared" si="7"/>
-        <v>31</v>
-      </c>
-      <c r="O26" s="7">
-        <f t="shared" si="8"/>
-        <v>39</v>
-      </c>
-      <c r="P26" s="5">
-        <f t="shared" si="9"/>
-        <v>19</v>
-      </c>
-      <c r="Q26" s="5">
-        <f t="shared" si="10"/>
-        <v>15</v>
-      </c>
-      <c r="R26" s="5">
-        <f t="shared" si="11"/>
-        <v>11</v>
-      </c>
-      <c r="S26" s="5">
-        <f t="shared" si="4"/>
-        <v>195</v>
-      </c>
-      <c r="T26" s="8">
-        <v>1</v>
-      </c>
-      <c r="U26" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="V26" t="s">
+      <c r="V25" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="27" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A26" s="1"/>
+      <c r="K26" s="19"/>
+      <c r="L26" s="31">
+        <f>SUM(L2:L11)+L20+SUM(L22:L24)</f>
+        <v>505</v>
+      </c>
+      <c r="M26" s="31">
+        <f>SUM(M2:M11)+M20+SUM(M22:M24)</f>
+        <v>692</v>
+      </c>
+      <c r="N26" s="31">
+        <f>SUM(N2:N11)+N20+SUM(N22:N24)</f>
+        <v>465</v>
+      </c>
+      <c r="O26" s="31">
+        <f>SUM(O2:O11)+O20+SUM(O22:O24)</f>
+        <v>527</v>
+      </c>
+      <c r="P26" s="31">
+        <f>SUM(P2:P11)+P20+SUM(P22:P24)</f>
+        <v>207</v>
+      </c>
+      <c r="Q26" s="31">
+        <f>SUM(Q2:Q11)+Q20+SUM(Q22:Q24)</f>
+        <v>292</v>
+      </c>
+      <c r="R26" s="31">
+        <f>SUM(R2:R11)+R20+SUM(R22:R24)</f>
+        <v>339</v>
+      </c>
+      <c r="S26" s="31">
+        <f>SUM(S2:S11)+S20+SUM(S22:S24)</f>
+        <v>3027</v>
+      </c>
+    </row>
+    <row r="27" spans="1:23" ht="11.4" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="1"/>
-      <c r="K27" s="19"/>
-      <c r="L27" s="31">
-        <f t="shared" ref="L27:S27" si="22">SUM(L2:L11)+L21+SUM(L23:L25)</f>
-        <v>505</v>
-      </c>
-      <c r="M27" s="31">
-        <f t="shared" si="22"/>
-        <v>692</v>
-      </c>
-      <c r="N27" s="31">
-        <f t="shared" si="22"/>
-        <v>465</v>
-      </c>
-      <c r="O27" s="31">
-        <f t="shared" si="22"/>
-        <v>527</v>
-      </c>
-      <c r="P27" s="31">
-        <f t="shared" si="22"/>
-        <v>207</v>
-      </c>
-      <c r="Q27" s="31">
-        <f t="shared" si="22"/>
-        <v>292</v>
-      </c>
-      <c r="R27" s="31">
-        <f t="shared" si="22"/>
-        <v>339</v>
-      </c>
-      <c r="S27" s="31">
-        <f t="shared" si="22"/>
-        <v>3027</v>
-      </c>
-    </row>
-    <row r="28" spans="1:23" ht="11.4" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="28" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A28" s="1"/>
     </row>
     <row r="29" spans="1:23" x14ac:dyDescent="0.25">
@@ -2586,9 +2560,6 @@
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A35" s="1"/>
-    </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A36" s="1"/>
     </row>
   </sheetData>
   <phoneticPr fontId="10" type="noConversion"/>

</xml_diff>